<commit_message>
fix(productos): Fase A — 8 guías «Cómo montar» y 10 planes de negocio v1.1: cache de valores, A4, metadata, bio anclada, versión; checklists OK con desplegable ✓/☐/N/A + fila verde + contador; referencias circulares reparadas (calculadora dark-kitchen ×12 celdas, cash-flow-break-even B12 ×5 guías) y 6 etiquetas «= …» que abrían con #¿NOMBRE? pasan a texto
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016924EP7QJuq6BNFj8S7Fks
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/guia-dark-kitchen/calculadora-viabilidad-dark-kitchen.xlsx
+++ b/astro-site/public/dl/guia-dark-kitchen/calculadora-viabilidad-dark-kitchen.xlsx
@@ -11,7 +11,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P&amp;L Mensual" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Punto de Equilibrio" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Inversión Inicial'!$4:$4</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -573,7 +575,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -599,6 +601,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1144,11 +1147,11 @@
       </c>
       <c r="C35" s="8">
         <f>SUM(C5:C34)</f>
-        <v/>
+        <v>57900.0</v>
       </c>
       <c r="D35" s="8">
         <f>SUM(D5:D34)</f>
-        <v/>
+        <v>0.0</v>
       </c>
     </row>
   </sheetData>
@@ -1156,7 +1159,16 @@
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;8 AI Chef Pro · aichef.pro · Página &amp;P de &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -1164,7 +1176,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:D35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1189,6 +1201,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -1256,6 +1269,8 @@
         <v>0.8</v>
       </c>
     </row>
+    <row r="11"/>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
@@ -1271,7 +1286,7 @@
       </c>
       <c r="B14" s="12">
         <f>B5*B6*B7</f>
-        <v/>
+        <v>23100.0</v>
       </c>
     </row>
     <row r="15">
@@ -1282,19 +1297,21 @@
       </c>
       <c r="B15" s="13">
         <f>-B5*B6*B7*B8</f>
-        <v/>
+        <v>-6930.0</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="9">
-        <f> Ingresos netos</f>
-        <v/>
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>= Ingresos netos</t>
+        </is>
       </c>
       <c r="B16" s="12">
         <f>B5*B6*B7*(1-B8)</f>
-        <v/>
-      </c>
-    </row>
+        <v>16169.999999999998</v>
+      </c>
+    </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
@@ -1303,7 +1320,7 @@
       </c>
       <c r="B18" s="13">
         <f>-B5*B6*B7*B9</f>
-        <v/>
+        <v>-6930.0</v>
       </c>
     </row>
     <row r="19">
@@ -1314,19 +1331,21 @@
       </c>
       <c r="B19" s="13">
         <f>-B5*B7*B10</f>
-        <v/>
+        <v>-840.0</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="9">
-        <f> Margen bruto</f>
-        <v/>
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>= Margen bruto</t>
+        </is>
       </c>
       <c r="B20" s="12">
         <f>B5*B6*B7*(1-B8-B9)-B5*B7*B10</f>
-        <v/>
-      </c>
-    </row>
+        <v>8400.0</v>
+      </c>
+    </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
@@ -1412,9 +1431,10 @@
       </c>
       <c r="B30" s="13">
         <f>B14*0.05</f>
-        <v/>
-      </c>
-    </row>
+        <v>1155.0</v>
+      </c>
+    </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
@@ -1423,9 +1443,10 @@
       </c>
       <c r="B32" s="14">
         <f>SUM(B23:B30)</f>
-        <v/>
-      </c>
-    </row>
+        <v>7585.0</v>
+      </c>
+    </row>
+    <row r="33"/>
     <row r="34">
       <c r="A34" s="15" t="inlineStr">
         <is>
@@ -1434,7 +1455,7 @@
       </c>
       <c r="B34" s="16">
         <f>B20-B32</f>
-        <v/>
+        <v>815.0</v>
       </c>
     </row>
     <row r="35">
@@ -1445,7 +1466,7 @@
       </c>
       <c r="B35" s="17">
         <f>IF(B14=0,0,B34/B14)</f>
-        <v/>
+        <v>0.03528138528138528</v>
       </c>
     </row>
   </sheetData>
@@ -1453,7 +1474,16 @@
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;8 AI Chef Pro · aichef.pro · Página &amp;P de &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -1461,7 +1491,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1487,6 +1517,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -1502,7 +1533,7 @@
       </c>
       <c r="B5" s="13">
         <f>'P&amp;L Mensual'!B6</f>
-        <v/>
+        <v>22.0</v>
       </c>
     </row>
     <row r="6">
@@ -1513,7 +1544,7 @@
       </c>
       <c r="B6" s="18">
         <f>'P&amp;L Mensual'!B8</f>
-        <v/>
+        <v>0.3</v>
       </c>
     </row>
     <row r="7">
@@ -1524,7 +1555,7 @@
       </c>
       <c r="B7" s="18">
         <f>'P&amp;L Mensual'!B9</f>
-        <v/>
+        <v>0.3</v>
       </c>
     </row>
     <row r="8">
@@ -1535,7 +1566,7 @@
       </c>
       <c r="B8" s="13">
         <f>'P&amp;L Mensual'!B10</f>
-        <v/>
+        <v>0.8</v>
       </c>
     </row>
     <row r="9">
@@ -1546,9 +1577,10 @@
       </c>
       <c r="B9" s="13">
         <f>'P&amp;L Mensual'!B32</f>
-        <v/>
-      </c>
-    </row>
+        <v>7585.0</v>
+      </c>
+    </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
@@ -1564,7 +1596,7 @@
       </c>
       <c r="B12" s="14">
         <f>B5*(1-B6-B7)-B8</f>
-        <v/>
+        <v>7.999999999999999</v>
       </c>
     </row>
     <row r="13">
@@ -1575,7 +1607,7 @@
       </c>
       <c r="B13" s="19">
         <f>ROUNDUP(B9/B12,0)</f>
-        <v/>
+        <v>949.0</v>
       </c>
     </row>
     <row r="14">
@@ -1586,7 +1618,7 @@
       </c>
       <c r="B14" s="19">
         <f>ROUNDUP(B13/30,0)</f>
-        <v/>
+        <v>32.0</v>
       </c>
     </row>
     <row r="15">
@@ -1597,9 +1629,11 @@
       </c>
       <c r="B15" s="20">
         <f>B13*B5</f>
-        <v/>
-      </c>
-    </row>
+        <v>20878.0</v>
+      </c>
+    </row>
+    <row r="16"/>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
@@ -1649,15 +1683,15 @@
       </c>
       <c r="B21" s="5">
         <f>B5</f>
-        <v/>
+        <v>22.0</v>
       </c>
       <c r="C21" s="5">
         <f>B5</f>
-        <v/>
+        <v>22.0</v>
       </c>
       <c r="D21" s="5">
         <f>B5</f>
-        <v/>
+        <v>22.0</v>
       </c>
     </row>
     <row r="22">
@@ -1668,15 +1702,15 @@
       </c>
       <c r="B22" s="12">
         <f>B20*B21*30</f>
-        <v/>
+        <v>13200.0</v>
       </c>
       <c r="C22" s="12">
         <f>C20*C21*30</f>
-        <v/>
+        <v>26400.0</v>
       </c>
       <c r="D22" s="12">
         <f>D20*D21*30</f>
-        <v/>
+        <v>42900.0</v>
       </c>
     </row>
     <row r="23">
@@ -1687,15 +1721,15 @@
       </c>
       <c r="B23" s="12">
         <f>-B22*B6</f>
-        <v/>
+        <v>-3960.0</v>
       </c>
       <c r="C23" s="12">
         <f>-C22*B6</f>
-        <v/>
+        <v>-7920.0</v>
       </c>
       <c r="D23" s="12">
         <f>-D22*B6</f>
-        <v/>
+        <v>-12870.0</v>
       </c>
     </row>
     <row r="24">
@@ -1705,16 +1739,16 @@
         </is>
       </c>
       <c r="B24" s="12">
-        <f>-B23*B7</f>
-        <v/>
+        <f>-B22*B7</f>
+        <v>-3960.0</v>
       </c>
       <c r="C24" s="12">
-        <f>-C23*B7</f>
-        <v/>
+        <f>-C22*B7</f>
+        <v>-7920.0</v>
       </c>
       <c r="D24" s="12">
-        <f>-D23*B7</f>
-        <v/>
+        <f>-D22*B7</f>
+        <v>-12870.0</v>
       </c>
     </row>
     <row r="25">
@@ -1725,33 +1759,34 @@
       </c>
       <c r="B25" s="12">
         <f>-B20*30*B8</f>
-        <v/>
+        <v>-480.0</v>
       </c>
       <c r="C25" s="12">
         <f>-C20*30*B8</f>
-        <v/>
+        <v>-960.0</v>
       </c>
       <c r="D25" s="12">
         <f>-D20*30*B8</f>
-        <v/>
+        <v>-1560.0</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="9">
-        <f> Margen bruto (€)</f>
-        <v/>
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>= Margen bruto (€)</t>
+        </is>
       </c>
       <c r="B26" s="12">
-        <f>SUM(B26:B29)</f>
-        <v/>
+        <f>SUM(B22:B25)</f>
+        <v>4800.0</v>
       </c>
       <c r="C26" s="12">
-        <f>SUM(C26:C29)</f>
-        <v/>
+        <f>SUM(C22:C25)</f>
+        <v>9600.0</v>
       </c>
       <c r="D26" s="12">
-        <f>SUM(D26:D29)</f>
-        <v/>
+        <f>SUM(D22:D25)</f>
+        <v>15600.0</v>
       </c>
     </row>
     <row r="27">
@@ -1762,33 +1797,34 @@
       </c>
       <c r="B27" s="12">
         <f>-B9</f>
-        <v/>
+        <v>-7585.0</v>
       </c>
       <c r="C27" s="12">
         <f>-B9</f>
-        <v/>
+        <v>-7585.0</v>
       </c>
       <c r="D27" s="12">
         <f>-B9</f>
-        <v/>
+        <v>-7585.0</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="9">
-        <f> EBITDA mensual (€)</f>
-        <v/>
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>= EBITDA mensual (€)</t>
+        </is>
       </c>
       <c r="B28" s="12">
-        <f>B32+B33</f>
-        <v/>
+        <f>B26+B27</f>
+        <v>-2785.0</v>
       </c>
       <c r="C28" s="12">
-        <f>C32+C33</f>
-        <v/>
+        <f>C26+C27</f>
+        <v>2015.0</v>
       </c>
       <c r="D28" s="12">
-        <f>D32+D33</f>
-        <v/>
+        <f>D26+D27</f>
+        <v>8015.0</v>
       </c>
     </row>
     <row r="29">
@@ -1798,16 +1834,16 @@
         </is>
       </c>
       <c r="B29" s="22">
-        <f>IF(B29=0,0,B35/B29)</f>
-        <v/>
+        <f>IF(B22=0,0,B28/B22)</f>
+        <v>-0.2109848484848485</v>
       </c>
       <c r="C29" s="22">
-        <f>IF(C29=0,0,C35/C29)</f>
-        <v/>
+        <f>IF(C22=0,0,C28/C22)</f>
+        <v>0.07632575757575757</v>
       </c>
       <c r="D29" s="22">
-        <f>IF(D29=0,0,D35/D29)</f>
-        <v/>
+        <f>IF(D22=0,0,D28/D22)</f>
+        <v>0.18682983682983684</v>
       </c>
     </row>
   </sheetData>
@@ -1815,6 +1851,15 @@
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;8 AI Chef Pro · aichef.pro · Página &amp;P de &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>